<commit_message>
Updated DEU model - 2025-09-07 11:48
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/vt_vervestacks_DEU_v1.xlsx
+++ b/VerveStacks_DEU/vt_vervestacks_DEU_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC4B93EC-0B20-4920-942F-C5B9837F2416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DC8E476-7935-4CDA-827D-872CB9961034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{C7B9D3CE-1739-4726-8687-322A540E8B38}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{A8EB2609-9AC4-4BD4-AE2F-1C425EEC7624}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -3383,7 +3383,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55FED866-F1F4-4C8C-8C22-6EA5460923A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC731AE5-A508-4BAF-BAEC-D585689EFB98}">
   <dimension ref="B9:T466"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -24562,7 +24562,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EFDACB6-7701-4FD5-B777-FC2ADE169747}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5900890F-FD68-4F15-8C10-80F07B936B91}">
   <dimension ref="B9:T623"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -48061,7 +48061,7 @@
         <v>33</v>
       </c>
       <c r="L525">
-        <v>0.14220084641443556</v>
+        <v>0.14220084641443553</v>
       </c>
     </row>
     <row r="526" spans="2:12" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Updated DEU model - 2025-09-07 18:25
</commit_message>
<xml_diff>
--- a/VerveStacks_DEU/vt_vervestacks_DEU_v1.xlsx
+++ b/VerveStacks_DEU/vt_vervestacks_DEU_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DEU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DC8E476-7935-4CDA-827D-872CB9961034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C21BB684-28A5-4F37-BC41-72961474FB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{A8EB2609-9AC4-4BD4-AE2F-1C425EEC7624}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{64CADF40-7A13-4854-BC94-E2DF6449C32F}"/>
   </bookViews>
   <sheets>
     <sheet name="ccs_retrofits" sheetId="2" r:id="rId1"/>
@@ -3383,7 +3383,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC731AE5-A508-4BAF-BAEC-D585689EFB98}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{357DCDFA-D6A3-4475-8BA8-0F98ACFE06B2}">
   <dimension ref="B9:T466"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -24562,7 +24562,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5900890F-FD68-4F15-8C10-80F07B936B91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F89970F-613B-4C4C-8212-44A8ED6C2C75}">
   <dimension ref="B9:T623"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
@@ -49099,7 +49099,7 @@
         <v>0.33123000000000002</v>
       </c>
       <c r="L555">
-        <v>0.55977485635294111</v>
+        <v>0.55977485635294122</v>
       </c>
     </row>
     <row r="556" spans="2:12" x14ac:dyDescent="0.45">
@@ -49904,7 +49904,7 @@
         <v>0.33123000000000002</v>
       </c>
       <c r="L590">
-        <v>0.33802250703984926</v>
+        <v>0.33802250703984932</v>
       </c>
     </row>
     <row r="591" spans="2:12" x14ac:dyDescent="0.45">

</xml_diff>